<commit_message>
db + seed sudah fix (done)
</commit_message>
<xml_diff>
--- a/backend/storage/imports/Master_SBM/13. SATUAN BIAYA PEMELIHARAAN DAN OPERASIONAL KENDARAAN DINAS.xlsx
+++ b/backend/storage/imports/Master_SBM/13. SATUAN BIAYA PEMELIHARAAN DAN OPERASIONAL KENDARAAN DINAS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\dokumen perkuliahan\kebutuhan magang\Projek magang\DITUGASKAN\SBM\baru 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UNIVERSITAS BINA SARANA INFORMATIKA(UBSI)\FILE MAGANG\Aplikasi Realisasi Keuangan\Relai\backend\storage\imports\Master_SBM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{362C143C-2965-4195-B2B9-DBE785CC9545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00644529-66CB-41B3-8C2A-E290C2870FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{51877813-44AA-4BD6-9165-B7815FC40D74}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="113">
   <si>
     <t>13.</t>
   </si>
@@ -397,6 +397,9 @@
       <t>PJR  RODA DUA
 (≥  750  CC)</t>
     </r>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -509,7 +512,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -554,12 +557,6 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
@@ -589,6 +586,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1003,14 +1003,18 @@
       <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="14">
-        <v>41277</v>
+      <c r="A7" s="14" t="s">
+        <v>112</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="17"/>
+      <c r="C7" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="D7" s="26" t="s">
+        <v>112</v>
+      </c>
       <c r="E7" s="12"/>
       <c r="F7" s="12"/>
     </row>
@@ -1600,10 +1604,10 @@
       <c r="C44" s="13">
         <v>-3</v>
       </c>
-      <c r="D44" s="18">
+      <c r="D44" s="16">
         <v>-4</v>
       </c>
-      <c r="E44" s="18">
+      <c r="E44" s="16">
         <v>-5</v>
       </c>
       <c r="F44" s="13">
@@ -1611,7 +1615,7 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="19">
+      <c r="A45" s="17">
         <v>1</v>
       </c>
       <c r="B45" s="2" t="s">
@@ -1631,7 +1635,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="19">
+      <c r="A46" s="17">
         <v>2</v>
       </c>
       <c r="B46" s="2" t="s">
@@ -1651,7 +1655,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="19">
+      <c r="A47" s="17">
         <v>3</v>
       </c>
       <c r="B47" s="2" t="s">
@@ -1671,7 +1675,7 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="19">
+      <c r="A48" s="17">
         <v>4</v>
       </c>
       <c r="B48" s="2" t="s">
@@ -1691,7 +1695,7 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="19">
+      <c r="A49" s="17">
         <v>5</v>
       </c>
       <c r="B49" s="2" t="s">
@@ -1711,7 +1715,7 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="19">
+      <c r="A50" s="17">
         <v>6</v>
       </c>
       <c r="B50" s="2" t="s">
@@ -1731,7 +1735,7 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="19">
+      <c r="A51" s="17">
         <v>7</v>
       </c>
       <c r="B51" s="2" t="s">
@@ -1751,7 +1755,7 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="19">
+      <c r="A52" s="17">
         <v>8</v>
       </c>
       <c r="B52" s="2" t="s">
@@ -1771,7 +1775,7 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="19">
+      <c r="A53" s="17">
         <v>9</v>
       </c>
       <c r="B53" s="2" t="s">
@@ -1791,7 +1795,7 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="19">
+      <c r="A54" s="17">
         <v>10</v>
       </c>
       <c r="B54" s="2" t="s">
@@ -1811,7 +1815,7 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="19">
+      <c r="A55" s="17">
         <v>11</v>
       </c>
       <c r="B55" s="2" t="s">
@@ -1831,7 +1835,7 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="19">
+      <c r="A56" s="17">
         <v>12</v>
       </c>
       <c r="B56" s="2" t="s">
@@ -1851,7 +1855,7 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="19">
+      <c r="A57" s="17">
         <v>13</v>
       </c>
       <c r="B57" s="2" t="s">
@@ -1871,7 +1875,7 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="19">
+      <c r="A58" s="17">
         <v>14</v>
       </c>
       <c r="B58" s="2" t="s">
@@ -1891,7 +1895,7 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="19">
+      <c r="A59" s="17">
         <v>15</v>
       </c>
       <c r="B59" s="2" t="s">
@@ -1911,7 +1915,7 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="19">
+      <c r="A60" s="17">
         <v>16</v>
       </c>
       <c r="B60" s="2" t="s">
@@ -1931,7 +1935,7 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="19">
+      <c r="A61" s="17">
         <v>17</v>
       </c>
       <c r="B61" s="2" t="s">
@@ -1951,7 +1955,7 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="19">
+      <c r="A62" s="17">
         <v>18</v>
       </c>
       <c r="B62" s="2" t="s">
@@ -1971,7 +1975,7 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="19">
+      <c r="A63" s="17">
         <v>19</v>
       </c>
       <c r="B63" s="2" t="s">
@@ -1991,7 +1995,7 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="19">
+      <c r="A64" s="17">
         <v>20</v>
       </c>
       <c r="B64" s="2" t="s">
@@ -2011,7 +2015,7 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="19">
+      <c r="A65" s="17">
         <v>21</v>
       </c>
       <c r="B65" s="2" t="s">
@@ -2031,7 +2035,7 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="19">
+      <c r="A66" s="17">
         <v>22</v>
       </c>
       <c r="B66" s="2" t="s">
@@ -2051,7 +2055,7 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="19">
+      <c r="A67" s="17">
         <v>23</v>
       </c>
       <c r="B67" s="2" t="s">
@@ -2071,7 +2075,7 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="19">
+      <c r="A68" s="17">
         <v>24</v>
       </c>
       <c r="B68" s="2" t="s">
@@ -2091,7 +2095,7 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="19">
+      <c r="A69" s="17">
         <v>25</v>
       </c>
       <c r="B69" s="2" t="s">
@@ -2111,7 +2115,7 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="19">
+      <c r="A70" s="17">
         <v>26</v>
       </c>
       <c r="B70" s="2" t="s">
@@ -2131,7 +2135,7 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="19">
+      <c r="A71" s="17">
         <v>27</v>
       </c>
       <c r="B71" s="2" t="s">
@@ -2151,7 +2155,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="19">
+      <c r="A72" s="17">
         <v>28</v>
       </c>
       <c r="B72" s="2" t="s">
@@ -2171,7 +2175,7 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="19">
+      <c r="A73" s="17">
         <v>29</v>
       </c>
       <c r="B73" s="2" t="s">
@@ -2191,7 +2195,7 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="19">
+      <c r="A74" s="17">
         <v>30</v>
       </c>
       <c r="B74" s="2" t="s">
@@ -2211,7 +2215,7 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="19">
+      <c r="A75" s="17">
         <v>31</v>
       </c>
       <c r="B75" s="2" t="s">
@@ -2231,7 +2235,7 @@
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="19">
+      <c r="A76" s="17">
         <v>32</v>
       </c>
       <c r="B76" s="2" t="s">
@@ -2251,7 +2255,7 @@
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="20">
+      <c r="A77" s="18">
         <v>33</v>
       </c>
       <c r="B77" s="2" t="s">
@@ -2271,7 +2275,7 @@
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="19">
+      <c r="A78" s="17">
         <v>34</v>
       </c>
       <c r="B78" s="2" t="s">
@@ -2297,10 +2301,10 @@
       <c r="B79" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C79" s="21"/>
-      <c r="D79" s="21"/>
-      <c r="E79" s="22"/>
-      <c r="F79" s="22"/>
+      <c r="C79" s="19"/>
+      <c r="D79" s="19"/>
+      <c r="E79" s="20"/>
+      <c r="F79" s="20"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
@@ -2309,20 +2313,20 @@
       <c r="B80" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="C80" s="23" t="s">
+      <c r="C80" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D80" s="23" t="s">
+      <c r="D80" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="E80" s="22"/>
-      <c r="F80" s="22"/>
+      <c r="E80" s="20"/>
+      <c r="F80" s="20"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="13">
         <v>-1</v>
       </c>
-      <c r="B81" s="18">
+      <c r="B81" s="16">
         <v>-2</v>
       </c>
       <c r="C81" s="13">
@@ -2331,72 +2335,72 @@
       <c r="D81" s="13">
         <v>-4</v>
       </c>
-      <c r="E81" s="22"/>
-      <c r="F81" s="22"/>
+      <c r="E81" s="20"/>
+      <c r="F81" s="20"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="19">
+      <c r="A82" s="17">
         <v>1</v>
       </c>
       <c r="B82" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="C82" s="24" t="s">
+      <c r="C82" s="22" t="s">
         <v>7</v>
       </c>
       <c r="D82" s="15">
         <v>9750000</v>
       </c>
-      <c r="E82" s="22"/>
-      <c r="F82" s="22"/>
+      <c r="E82" s="20"/>
+      <c r="F82" s="20"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="19">
+      <c r="A83" s="17">
         <v>2</v>
       </c>
       <c r="B83" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="C83" s="24" t="s">
+      <c r="C83" s="22" t="s">
         <v>7</v>
       </c>
       <c r="D83" s="15">
         <v>37110000</v>
       </c>
-      <c r="E83" s="22"/>
-      <c r="F83" s="22"/>
+      <c r="E83" s="20"/>
+      <c r="F83" s="20"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="19">
+      <c r="A84" s="17">
         <v>3</v>
       </c>
       <c r="B84" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="C84" s="24" t="s">
+      <c r="C84" s="22" t="s">
         <v>7</v>
       </c>
       <c r="D84" s="15">
         <v>40760000</v>
       </c>
-      <c r="E84" s="22"/>
-      <c r="F84" s="22"/>
+      <c r="E84" s="20"/>
+      <c r="F84" s="20"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="19">
+      <c r="A85" s="17">
         <v>4</v>
       </c>
       <c r="B85" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="C85" s="24" t="s">
+      <c r="C85" s="22" t="s">
         <v>7</v>
       </c>
       <c r="D85" s="15">
         <v>20240000</v>
       </c>
-      <c r="E85" s="22"/>
-      <c r="F85" s="22"/>
+      <c r="E85" s="20"/>
+      <c r="F85" s="20"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="10">
@@ -2423,10 +2427,10 @@
       <c r="D87" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E87" s="25" t="s">
+      <c r="E87" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="F87" s="25" t="s">
+      <c r="F87" s="23" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2451,7 +2455,7 @@
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="19">
+      <c r="A89" s="17">
         <v>1</v>
       </c>
       <c r="B89" s="2" t="s">
@@ -2460,18 +2464,18 @@
       <c r="C89" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D89" s="26">
+      <c r="D89" s="24">
         <v>78370000</v>
       </c>
-      <c r="E89" s="26">
+      <c r="E89" s="24">
         <v>19680000</v>
       </c>
-      <c r="F89" s="26">
+      <c r="F89" s="24">
         <v>47080000</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="19">
+      <c r="A90" s="17">
         <v>2</v>
       </c>
       <c r="B90" s="2" t="s">
@@ -2480,18 +2484,18 @@
       <c r="C90" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D90" s="26">
+      <c r="D90" s="24">
         <v>75920000</v>
       </c>
-      <c r="E90" s="26">
+      <c r="E90" s="24">
         <v>18960000</v>
       </c>
-      <c r="F90" s="26">
+      <c r="F90" s="24">
         <v>43840000</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="19">
+      <c r="A91" s="17">
         <v>3</v>
       </c>
       <c r="B91" s="2" t="s">
@@ -2500,18 +2504,18 @@
       <c r="C91" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D91" s="26">
+      <c r="D91" s="24">
         <v>76090000</v>
       </c>
-      <c r="E91" s="26">
+      <c r="E91" s="24">
         <v>18890000</v>
       </c>
-      <c r="F91" s="26">
+      <c r="F91" s="24">
         <v>42510000</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="19">
+      <c r="A92" s="17">
         <v>4</v>
       </c>
       <c r="B92" s="2" t="s">
@@ -2520,18 +2524,18 @@
       <c r="C92" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D92" s="26">
+      <c r="D92" s="24">
         <v>75650000</v>
       </c>
-      <c r="E92" s="26">
+      <c r="E92" s="24">
         <v>18580000</v>
       </c>
-      <c r="F92" s="26">
+      <c r="F92" s="24">
         <v>40750000</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="19">
+      <c r="A93" s="17">
         <v>5</v>
       </c>
       <c r="B93" s="2" t="s">
@@ -2540,18 +2544,18 @@
       <c r="C93" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D93" s="26">
+      <c r="D93" s="24">
         <v>77330000</v>
       </c>
-      <c r="E93" s="26">
+      <c r="E93" s="24">
         <v>19310000</v>
       </c>
-      <c r="F93" s="26">
+      <c r="F93" s="24">
         <v>44930000</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="19">
+      <c r="A94" s="17">
         <v>6</v>
       </c>
       <c r="B94" s="2" t="s">
@@ -2560,18 +2564,18 @@
       <c r="C94" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D94" s="26">
+      <c r="D94" s="24">
         <v>77250000</v>
       </c>
-      <c r="E94" s="26">
+      <c r="E94" s="24">
         <v>19450000</v>
       </c>
-      <c r="F94" s="26">
+      <c r="F94" s="24">
         <v>46750000</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="19">
+      <c r="A95" s="17">
         <v>7</v>
       </c>
       <c r="B95" s="2" t="s">
@@ -2580,18 +2584,18 @@
       <c r="C95" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D95" s="26">
+      <c r="D95" s="24">
         <v>76130000</v>
       </c>
-      <c r="E95" s="26">
+      <c r="E95" s="24">
         <v>18880000</v>
       </c>
-      <c r="F95" s="26">
+      <c r="F95" s="24">
         <v>42480000</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="19">
+      <c r="A96" s="17">
         <v>8</v>
       </c>
       <c r="B96" s="2" t="s">
@@ -2600,18 +2604,18 @@
       <c r="C96" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D96" s="26">
+      <c r="D96" s="24">
         <v>76340000</v>
       </c>
-      <c r="E96" s="26">
+      <c r="E96" s="24">
         <v>18960000</v>
       </c>
-      <c r="F96" s="26">
+      <c r="F96" s="24">
         <v>42900000</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="19">
+      <c r="A97" s="17">
         <v>9</v>
       </c>
       <c r="B97" s="2" t="s">
@@ -2620,18 +2624,18 @@
       <c r="C97" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D97" s="26">
+      <c r="D97" s="24">
         <v>76180000</v>
       </c>
-      <c r="E97" s="26">
+      <c r="E97" s="24">
         <v>18900000</v>
       </c>
-      <c r="F97" s="26">
+      <c r="F97" s="24">
         <v>42570000</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="19">
+      <c r="A98" s="17">
         <v>10</v>
       </c>
       <c r="B98" s="2" t="s">
@@ -2640,18 +2644,18 @@
       <c r="C98" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D98" s="26">
+      <c r="D98" s="24">
         <v>75620000</v>
       </c>
-      <c r="E98" s="26">
+      <c r="E98" s="24">
         <v>18700000</v>
       </c>
-      <c r="F98" s="26">
+      <c r="F98" s="24">
         <v>41420000</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="19">
+      <c r="A99" s="17">
         <v>11</v>
       </c>
       <c r="B99" s="2" t="s">
@@ -2660,18 +2664,18 @@
       <c r="C99" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D99" s="26">
+      <c r="D99" s="24">
         <v>75790000</v>
       </c>
-      <c r="E99" s="26">
+      <c r="E99" s="24">
         <v>18580000</v>
       </c>
-      <c r="F99" s="26">
+      <c r="F99" s="24">
         <v>40820000</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="19">
+      <c r="A100" s="17">
         <v>12</v>
       </c>
       <c r="B100" s="2" t="s">
@@ -2680,18 +2684,18 @@
       <c r="C100" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D100" s="26">
+      <c r="D100" s="24">
         <v>75650000</v>
       </c>
-      <c r="E100" s="26">
+      <c r="E100" s="24">
         <v>18530000</v>
       </c>
-      <c r="F100" s="26">
+      <c r="F100" s="24">
         <v>40540000</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="19">
+      <c r="A101" s="17">
         <v>13</v>
       </c>
       <c r="B101" s="2" t="s">
@@ -2700,18 +2704,18 @@
       <c r="C101" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D101" s="26">
+      <c r="D101" s="24">
         <v>76300000</v>
       </c>
-      <c r="E101" s="26">
+      <c r="E101" s="24">
         <v>18800000</v>
       </c>
-      <c r="F101" s="26">
+      <c r="F101" s="24">
         <v>42060000</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="19">
+      <c r="A102" s="17">
         <v>14</v>
       </c>
       <c r="B102" s="2" t="s">
@@ -2720,18 +2724,18 @@
       <c r="C102" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D102" s="26">
+      <c r="D102" s="24">
         <v>78910000</v>
       </c>
-      <c r="E102" s="26">
+      <c r="E102" s="24">
         <v>19750000</v>
       </c>
-      <c r="F102" s="26">
+      <c r="F102" s="24">
         <v>47550000</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="19">
+      <c r="A103" s="17">
         <v>15</v>
       </c>
       <c r="B103" s="2" t="s">
@@ -2740,18 +2744,18 @@
       <c r="C103" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D103" s="26">
+      <c r="D103" s="24">
         <v>78490000</v>
       </c>
-      <c r="E103" s="26">
+      <c r="E103" s="24">
         <v>19610000</v>
       </c>
-      <c r="F103" s="26">
+      <c r="F103" s="24">
         <v>46700000</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="19">
+      <c r="A104" s="17">
         <v>16</v>
       </c>
       <c r="B104" s="2" t="s">
@@ -2760,18 +2764,18 @@
       <c r="C104" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D104" s="26">
+      <c r="D104" s="24">
         <v>76190000</v>
       </c>
-      <c r="E104" s="26">
+      <c r="E104" s="24">
         <v>18800000</v>
       </c>
-      <c r="F104" s="26">
+      <c r="F104" s="24">
         <v>42050000</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="19">
+      <c r="A105" s="17">
         <v>17</v>
       </c>
       <c r="B105" s="2" t="s">
@@ -2780,18 +2784,18 @@
       <c r="C105" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D105" s="26">
+      <c r="D105" s="24">
         <v>79630000</v>
       </c>
-      <c r="E105" s="26">
+      <c r="E105" s="24">
         <v>20250000</v>
       </c>
-      <c r="F105" s="26">
+      <c r="F105" s="24">
         <v>51490000</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="19">
+      <c r="A106" s="17">
         <v>18</v>
       </c>
       <c r="B106" s="2" t="s">
@@ -2800,18 +2804,18 @@
       <c r="C106" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D106" s="26">
+      <c r="D106" s="24">
         <v>77160000</v>
       </c>
-      <c r="E106" s="26">
+      <c r="E106" s="24">
         <v>19310000</v>
       </c>
-      <c r="F106" s="26">
+      <c r="F106" s="24">
         <v>45930000</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="19">
+      <c r="A107" s="17">
         <v>19</v>
       </c>
       <c r="B107" s="2" t="s">
@@ -2820,18 +2824,18 @@
       <c r="C107" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D107" s="26">
+      <c r="D107" s="24">
         <v>75210000</v>
       </c>
-      <c r="E107" s="26">
+      <c r="E107" s="24">
         <v>18610000</v>
       </c>
-      <c r="F107" s="26">
+      <c r="F107" s="24">
         <v>41760000</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="19">
+      <c r="A108" s="17">
         <v>20</v>
       </c>
       <c r="B108" s="2" t="s">
@@ -2840,18 +2844,18 @@
       <c r="C108" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D108" s="26">
+      <c r="D108" s="24">
         <v>77390000</v>
       </c>
-      <c r="E108" s="26">
+      <c r="E108" s="24">
         <v>19140000</v>
       </c>
-      <c r="F108" s="26">
+      <c r="F108" s="24">
         <v>44860000</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="19">
+      <c r="A109" s="17">
         <v>21</v>
       </c>
       <c r="B109" s="2" t="s">
@@ -2860,18 +2864,18 @@
       <c r="C109" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D109" s="26">
+      <c r="D109" s="24">
         <v>80690000</v>
       </c>
-      <c r="E109" s="26">
+      <c r="E109" s="24">
         <v>20370000</v>
       </c>
-      <c r="F109" s="26">
+      <c r="F109" s="24">
         <v>52090000</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="19">
+      <c r="A110" s="17">
         <v>22</v>
       </c>
       <c r="B110" s="2" t="s">
@@ -2880,18 +2884,18 @@
       <c r="C110" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D110" s="26">
+      <c r="D110" s="24">
         <v>77840000</v>
       </c>
-      <c r="E110" s="26">
+      <c r="E110" s="24">
         <v>19280000</v>
       </c>
-      <c r="F110" s="26">
+      <c r="F110" s="24">
         <v>45680000</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="19">
+      <c r="A111" s="17">
         <v>23</v>
       </c>
       <c r="B111" s="2" t="s">
@@ -2900,18 +2904,18 @@
       <c r="C111" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D111" s="26">
+      <c r="D111" s="24">
         <v>77060000</v>
       </c>
-      <c r="E111" s="26">
+      <c r="E111" s="24">
         <v>18980000</v>
       </c>
-      <c r="F111" s="26">
+      <c r="F111" s="24">
         <v>43890000</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="19">
+      <c r="A112" s="17">
         <v>24</v>
       </c>
       <c r="B112" s="2" t="s">
@@ -2920,18 +2924,18 @@
       <c r="C112" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D112" s="26">
+      <c r="D112" s="24">
         <v>76310000</v>
       </c>
-      <c r="E112" s="26">
+      <c r="E112" s="24">
         <v>18720000</v>
       </c>
-      <c r="F112" s="26">
+      <c r="F112" s="24">
         <v>42370000</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="19">
+      <c r="A113" s="17">
         <v>25</v>
       </c>
       <c r="B113" s="2" t="s">
@@ -2940,18 +2944,18 @@
       <c r="C113" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D113" s="26">
+      <c r="D113" s="24">
         <v>76890000</v>
       </c>
-      <c r="E113" s="26">
+      <c r="E113" s="24">
         <v>18990000</v>
       </c>
-      <c r="F113" s="26">
+      <c r="F113" s="24">
         <v>43960000</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A114" s="19">
+      <c r="A114" s="17">
         <v>26</v>
       </c>
       <c r="B114" s="2" t="s">
@@ -2960,18 +2964,18 @@
       <c r="C114" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D114" s="26">
+      <c r="D114" s="24">
         <v>76330000</v>
       </c>
-      <c r="E114" s="26">
+      <c r="E114" s="24">
         <v>18880000</v>
       </c>
-      <c r="F114" s="26">
+      <c r="F114" s="24">
         <v>43280000</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" s="19">
+      <c r="A115" s="17">
         <v>27</v>
       </c>
       <c r="B115" s="2" t="s">
@@ -2980,18 +2984,18 @@
       <c r="C115" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D115" s="26">
+      <c r="D115" s="24">
         <v>73760000</v>
       </c>
-      <c r="E115" s="26">
+      <c r="E115" s="24">
         <v>17910000</v>
       </c>
-      <c r="F115" s="26">
+      <c r="F115" s="24">
         <v>36890000</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" s="19">
+      <c r="A116" s="17">
         <v>28</v>
       </c>
       <c r="B116" s="2" t="s">
@@ -3000,18 +3004,18 @@
       <c r="C116" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D116" s="26">
+      <c r="D116" s="24">
         <v>76260000</v>
       </c>
-      <c r="E116" s="26">
+      <c r="E116" s="24">
         <v>18770000</v>
       </c>
-      <c r="F116" s="26">
+      <c r="F116" s="24">
         <v>41870000</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" s="19">
+      <c r="A117" s="17">
         <v>29</v>
       </c>
       <c r="B117" s="2" t="s">
@@ -3020,18 +3024,18 @@
       <c r="C117" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D117" s="26">
+      <c r="D117" s="24">
         <v>78000000</v>
       </c>
-      <c r="E117" s="26">
+      <c r="E117" s="24">
         <v>19410000</v>
       </c>
-      <c r="F117" s="26">
+      <c r="F117" s="24">
         <v>46420000</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" s="19">
+      <c r="A118" s="17">
         <v>30</v>
       </c>
       <c r="B118" s="2" t="s">
@@ -3040,18 +3044,18 @@
       <c r="C118" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D118" s="26">
+      <c r="D118" s="24">
         <v>78920000</v>
       </c>
-      <c r="E118" s="26">
+      <c r="E118" s="24">
         <v>19710000</v>
       </c>
-      <c r="F118" s="26">
+      <c r="F118" s="24">
         <v>48200000</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="19">
+      <c r="A119" s="17">
         <v>31</v>
       </c>
       <c r="B119" s="2" t="s">
@@ -3060,18 +3064,18 @@
       <c r="C119" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D119" s="26">
+      <c r="D119" s="24">
         <v>78230000</v>
       </c>
-      <c r="E119" s="26">
+      <c r="E119" s="24">
         <v>19710000</v>
       </c>
-      <c r="F119" s="26">
+      <c r="F119" s="24">
         <v>47080000</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="19">
+      <c r="A120" s="17">
         <v>32</v>
       </c>
       <c r="B120" s="2" t="s">
@@ -3080,18 +3084,18 @@
       <c r="C120" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D120" s="26">
+      <c r="D120" s="24">
         <v>76510000</v>
       </c>
-      <c r="E120" s="26">
+      <c r="E120" s="24">
         <v>19160000</v>
       </c>
-      <c r="F120" s="26">
+      <c r="F120" s="24">
         <v>43940000</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" s="20">
+      <c r="A121" s="18">
         <v>33</v>
       </c>
       <c r="B121" s="2" t="s">
@@ -3100,18 +3104,18 @@
       <c r="C121" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D121" s="26">
+      <c r="D121" s="24">
         <v>77590000</v>
       </c>
-      <c r="E121" s="26">
+      <c r="E121" s="24">
         <v>19900000</v>
       </c>
-      <c r="F121" s="26">
+      <c r="F121" s="24">
         <v>48090000</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="19">
+      <c r="A122" s="17">
         <v>34</v>
       </c>
       <c r="B122" s="2" t="s">
@@ -3120,13 +3124,13 @@
       <c r="C122" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D122" s="26">
+      <c r="D122" s="24">
         <v>77690000</v>
       </c>
-      <c r="E122" s="26">
+      <c r="E122" s="24">
         <v>19640000</v>
       </c>
-      <c r="F122" s="26">
+      <c r="F122" s="24">
         <v>46680000</v>
       </c>
     </row>
@@ -3139,8 +3143,8 @@
       </c>
       <c r="C123" s="6"/>
       <c r="D123" s="6"/>
-      <c r="E123" s="27"/>
-      <c r="F123" s="27"/>
+      <c r="E123" s="25"/>
+      <c r="F123" s="25"/>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
@@ -3155,14 +3159,14 @@
       <c r="D124" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E124" s="27"/>
-      <c r="F124" s="27"/>
+      <c r="E124" s="25"/>
+      <c r="F124" s="25"/>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="13">
         <v>-1</v>
       </c>
-      <c r="B125" s="18">
+      <c r="B125" s="16">
         <v>-2</v>
       </c>
       <c r="C125" s="13">
@@ -3171,11 +3175,11 @@
       <c r="D125" s="13">
         <v>-4</v>
       </c>
-      <c r="E125" s="27"/>
-      <c r="F125" s="27"/>
+      <c r="E125" s="25"/>
+      <c r="F125" s="25"/>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" s="19">
+      <c r="A126" s="17">
         <v>1</v>
       </c>
       <c r="B126" s="7" t="s">
@@ -3187,11 +3191,11 @@
       <c r="D126" s="9">
         <v>35000000</v>
       </c>
-      <c r="E126" s="27"/>
-      <c r="F126" s="27"/>
+      <c r="E126" s="25"/>
+      <c r="F126" s="25"/>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" s="19">
+      <c r="A127" s="17">
         <v>2</v>
       </c>
       <c r="B127" s="7" t="s">
@@ -3203,11 +3207,11 @@
       <c r="D127" s="9">
         <v>33800000</v>
       </c>
-      <c r="E127" s="27"/>
-      <c r="F127" s="27"/>
+      <c r="E127" s="25"/>
+      <c r="F127" s="25"/>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" s="19">
+      <c r="A128" s="17">
         <v>3</v>
       </c>
       <c r="B128" s="7" t="s">
@@ -3219,8 +3223,8 @@
       <c r="D128" s="9">
         <v>30000000</v>
       </c>
-      <c r="E128" s="27"/>
-      <c r="F128" s="27"/>
+      <c r="E128" s="25"/>
+      <c r="F128" s="25"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="10">
@@ -3231,8 +3235,8 @@
       </c>
       <c r="C129" s="6"/>
       <c r="D129" s="6"/>
-      <c r="E129" s="27"/>
-      <c r="F129" s="27"/>
+      <c r="E129" s="25"/>
+      <c r="F129" s="25"/>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
@@ -3247,14 +3251,14 @@
       <c r="D130" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E130" s="27"/>
-      <c r="F130" s="27"/>
+      <c r="E130" s="25"/>
+      <c r="F130" s="25"/>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="13">
         <v>-1</v>
       </c>
-      <c r="B131" s="18">
+      <c r="B131" s="16">
         <v>-2</v>
       </c>
       <c r="C131" s="13">
@@ -3263,11 +3267,11 @@
       <c r="D131" s="13">
         <v>-4</v>
       </c>
-      <c r="E131" s="27"/>
-      <c r="F131" s="27"/>
+      <c r="E131" s="25"/>
+      <c r="F131" s="25"/>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="19">
+      <c r="A132" s="17">
         <v>1</v>
       </c>
       <c r="B132" s="7" t="s">
@@ -3279,11 +3283,11 @@
       <c r="D132" s="9">
         <v>14840000</v>
       </c>
-      <c r="E132" s="27"/>
-      <c r="F132" s="27"/>
+      <c r="E132" s="25"/>
+      <c r="F132" s="25"/>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="19">
+      <c r="A133" s="17">
         <v>2</v>
       </c>
       <c r="B133" s="7" t="s">
@@ -3295,11 +3299,11 @@
       <c r="D133" s="9">
         <v>11100000</v>
       </c>
-      <c r="E133" s="27"/>
-      <c r="F133" s="27"/>
+      <c r="E133" s="25"/>
+      <c r="F133" s="25"/>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="19">
+      <c r="A134" s="17">
         <v>3</v>
       </c>
       <c r="B134" s="7" t="s">
@@ -3311,11 +3315,11 @@
       <c r="D134" s="9">
         <v>10990000</v>
       </c>
-      <c r="E134" s="27"/>
-      <c r="F134" s="27"/>
+      <c r="E134" s="25"/>
+      <c r="F134" s="25"/>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="19">
+      <c r="A135" s="17">
         <v>4</v>
       </c>
       <c r="B135" s="7" t="s">
@@ -3327,11 +3331,11 @@
       <c r="D135" s="9">
         <v>10460000</v>
       </c>
-      <c r="E135" s="27"/>
-      <c r="F135" s="27"/>
+      <c r="E135" s="25"/>
+      <c r="F135" s="25"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="19">
+      <c r="A136" s="17">
         <v>5</v>
       </c>
       <c r="B136" s="7" t="s">
@@ -3343,8 +3347,8 @@
       <c r="D136" s="9">
         <v>3200000</v>
       </c>
-      <c r="E136" s="27"/>
-      <c r="F136" s="27"/>
+      <c r="E136" s="25"/>
+      <c r="F136" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>